<commit_message>
feat(uk2): dashboard UK-2, README, perbaikan expected & kebocoran path
- web/uk2.html + uk2.js: dashboard UK-2 (produk + 3 sampel materi): verifikasi,
  matriks skenario, test case (filter), ruang parameter, telaah metode, expected,
  pemetaan hasil, keterlacakan; navigasi UK-2 aktif di semua halaman
- expected: PR-K-02 → AES-256-GCM (Wycheproof), KAT HKDF ← RFC 8448, SHAKE256 batas
- context: path UK-1 relatif (tidak membocorkan path lokal) + test kebocoran
- README bagian UK-2 (peta KUK, cara menjalankan, PERLU_VERIFIKASI, saran UK-3);
  requirements (python-pptx, jsonschema), Makefile (uk2, uk2-samples), CI

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/uk2/test_cases.xlsx
+++ b/outputs/uk2/test_cases.xlsx
@@ -1719,7 +1719,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>COCOK_VEKTOR_RESMI; PERLU_VERIFIKASI</t>
+          <t>COCOK_VEKTOR_RESMI</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>COCOK_VEKTOR_RESMI; PERLU_VERIFIKASI</t>
+          <t>COCOK_VEKTOR_RESMI</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>BLAKE2B-512; SHA-1; SHA-256; SHA-384; SHA-512/256; SHA3-256; SHAKE256; HMAC-SHA-256-K128; HMAC-SHA-256-K256</t>
+          <t>BLAKE2B-512; SHA-1; SHA-256; SHA-384; SHA-512/256; SHA3-256; SHAKE256</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Objek uji tersedia &amp; terkonfigurasi: BLAKE2B-512, SHA-1, SHA-256, SHA-384, SHA-512/256, SHA3-256, SHAKE256, HMAC-SHA-256-K128 … | Kunci &amp; data uji ilustratif (bukan material produksi) | Fitur/akses tersedia: streaming_api | Expected value terverifikasi integritasnya (SHA-256 berkas expected/*.json)</t>
+          <t>Objek uji tersedia &amp; terkonfigurasi: BLAKE2B-512, SHA-1, SHA-256, SHA-384, SHA-512/256, SHA3-256, SHAKE256 | Kunci &amp; data uji ilustratif (bukan material produksi) | Fitur/akses tersedia: streaming_api | Expected value terverifikasi integritasnya (SHA-256 berkas expected/*.json)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>COCOK_VEKTOR_RESMI; PERLU_VERIFIKASI</t>
+          <t>COCOK_VEKTOR_RESMI</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>COCOK_VEKTOR_RESMI; PERLU_VERIFIKASI</t>
+          <t>COCOK_VEKTOR_RESMI</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">

</xml_diff>